<commit_message>
New changes banking flow
</commit_message>
<xml_diff>
--- a/test-data/userDataTDL.xlsx
+++ b/test-data/userDataTDL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/priyanshu/PROJECTS/Playwright_Automation/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{259EB670-F9C2-164D-A171-832AC2F7AC48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{387D467C-D3F6-9D4C-B894-CA4C13F2C689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="16">
   <si>
     <t>executor</t>
   </si>
@@ -31,23 +31,59 @@
     <t>Request_id</t>
   </si>
   <si>
-    <t>01</t>
-  </si>
-  <si>
     <t>Y</t>
   </si>
   <si>
-    <t>02</t>
+    <t>09</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>TC01</t>
+  </si>
+  <si>
+    <t>TC02</t>
+  </si>
+  <si>
+    <t>TC03</t>
+  </si>
+  <si>
+    <t>TC04</t>
+  </si>
+  <si>
+    <t>TC05</t>
+  </si>
+  <si>
+    <t>TC06</t>
+  </si>
+  <si>
+    <t>TC07</t>
+  </si>
+  <si>
+    <t>TC08</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -414,7 +450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -430,24 +466,97 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
         <v>5</v>
       </c>
     </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C1 B2 B3" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:C1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
new changes fro jenkins
</commit_message>
<xml_diff>
--- a/test-data/userDataTDL.xlsx
+++ b/test-data/userDataTDL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/priyanshu/PROJECTS/Playwright_Automation/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{387D467C-D3F6-9D4C-B894-CA4C13F2C689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{396EFDC3-A0A6-E144-BA2F-AD8861A0215C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -474,7 +474,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
@@ -482,7 +482,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
         <v>10</v>
@@ -490,7 +490,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>

</xml_diff>